<commit_message>
fixes en ISIN als basis
</commit_message>
<xml_diff>
--- a/.gitignore/Nieuw - Microsoft Excel Worksheet.xlsx
+++ b/.gitignore/Nieuw - Microsoft Excel Worksheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gwenh\Documenten\GitHub\Homeassistant-portfolio-tracker\.gitignore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{911AD6EE-90F0-40FC-B9E3-99C538270538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10FC693-F4CF-4380-8547-87630331B78A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,22 +25,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>fout op portefeuille boeking</t>
+    <t>fout op asset creatie warrant</t>
+  </si>
+  <si>
+    <t>ook voor het fotomoment geen waarde:</t>
+  </si>
+  <si>
+    <t>enkel volgende loggings:</t>
+  </si>
+  <si>
+    <t>_bf_request(instrument_information): HTTP 403 blijft na verse salt (salt=dynamisch) |  — Börse Frankfurt 30s gepauzeerd (poging 1)</t>
+  </si>
+  <si>
+    <t>_bf_request(instrument_information): HTTP 403 blijft na verse salt (salt=dynamisch) |  — Börse Frankfurt 60s gepauzeerd (poging 2)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF141414"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,8 +80,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -87,22 +107,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>135218</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>28978</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>135155</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>48615</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE8DDA62-2AAC-4FEE-82DB-B0F52F78FC33}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A94E9616-D028-453B-B9DE-751D40685E29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -118,8 +138,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="161925" y="762000"/>
-          <a:ext cx="13384493" cy="2886478"/>
+          <a:off x="0" y="571500"/>
+          <a:ext cx="12936755" cy="7097115"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -132,21 +152,21 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>325682</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>152714</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>48312</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>57424</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="5" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F297FE4E-AE35-41A3-B0F5-50279D893F78}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8B6662F-4323-4833-A872-1053D100E12B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -162,8 +182,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="3810000"/>
-          <a:ext cx="13127282" cy="2248214"/>
+          <a:off x="0" y="8001000"/>
+          <a:ext cx="4925112" cy="1962424"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -438,16 +458,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:A56"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>